<commit_message>
adverb annotation + optimization
</commit_message>
<xml_diff>
--- a/physical_location_labelling/physical_location_by_context/results/v03_gpt_annotation/kohad_1000_gpt_valjund_excel.xlsx
+++ b/physical_location_labelling/physical_location_by_context/results/v03_gpt_annotation/kohad_1000_gpt_valjund_excel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eestikeeleinstituut-my.sharepoint.com/personal/kertu_saul_eki_ee/Documents/Dokumendid/doktoritoo/estnltk_syntax_repo_kloon/physical_location_labelling/physical_location_by_context/results/v03_gpt_annotation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="332" documentId="8_{BEC30906-46EE-4C43-A66A-D354C8275BEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EF69073-3BCF-47DC-BC99-4553D597AB10}"/>
+  <xr:revisionPtr revIDLastSave="347" documentId="8_{BEC30906-46EE-4C43-A66A-D354C8275BEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15E3BC23-A76D-43AC-8998-DC660DE8536C}"/>
   <bookViews>
-    <workbookView xWindow="2013" yWindow="3140" windowWidth="19200" windowHeight="10073" activeTab="1" xr2:uid="{C390DCA3-6CE8-4683-AFF8-BA98244D7D99}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13986" firstSheet="1" activeTab="4" xr2:uid="{C390DCA3-6CE8-4683-AFF8-BA98244D7D99}"/>
   </bookViews>
   <sheets>
     <sheet name="kohad_1000_gpt_väljund" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId8"/>
     <pivotCache cacheId="1" r:id="rId9"/>
-    <pivotCache cacheId="21" r:id="rId10"/>
+    <pivotCache cacheId="2" r:id="rId10"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7705" uniqueCount="2027">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7706" uniqueCount="2028">
   <si>
     <t>lause</t>
   </si>
@@ -6139,6 +6139,9 @@
   </si>
   <si>
     <t>name</t>
+  </si>
+  <si>
+    <t>Kokku</t>
   </si>
 </sst>
 </file>
@@ -6233,7 +6236,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -6252,17 +6255,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -17458,7 +17450,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E59E14F4-8CD2-48C7-B185-F8FA9ED16BBE}" name="PivotTable10" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E59E14F4-8CD2-48C7-B185-F8FA9ED16BBE}" name="PivotTable10" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="1">
   <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -17592,19 +17584,9 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1D7FD598-83F9-4867-9985-8FD53BDEED42}" name="Table5" displayName="Table5" ref="A1:E1001" totalsRowShown="0">
   <autoFilter ref="A1:E1001" xr:uid="{1D7FD598-83F9-4867-9985-8FD53BDEED42}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="NONE"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="3">
-      <filters>
-        <filter val="loc_c"/>
-      </filters>
-    </filterColumn>
     <filterColumn colId="4">
       <filters>
-        <filter val="name"/>
+        <filter val="org"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -29159,7 +29141,7 @@
         <v>2007</v>
       </c>
     </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
@@ -29176,7 +29158,7 @@
         <v>2015</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A15" s="1" t="s">
         <v>30</v>
       </c>
@@ -30213,7 +30195,7 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="88" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
+    <row r="88" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
       <c r="A88" s="1" t="s">
         <v>174</v>
       </c>
@@ -30965,7 +30947,7 @@
         <v>2009</v>
       </c>
     </row>
-    <row r="140" spans="1:5" ht="43" hidden="1" x14ac:dyDescent="0.5">
+    <row r="140" spans="1:5" ht="43" x14ac:dyDescent="0.5">
       <c r="A140" s="1" t="s">
         <v>276</v>
       </c>
@@ -31167,7 +31149,7 @@
         <v>2009</v>
       </c>
     </row>
-    <row r="154" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
+    <row r="154" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A154" s="1" t="s">
         <v>304</v>
       </c>
@@ -31862,7 +31844,7 @@
         <v>2009</v>
       </c>
     </row>
-    <row r="203" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A203" s="1" t="s">
         <v>402</v>
       </c>
@@ -31921,7 +31903,7 @@
         <v>2003</v>
       </c>
     </row>
-    <row r="207" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A207" s="1" t="s">
         <v>410</v>
       </c>
@@ -33272,7 +33254,7 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="302" spans="1:5" ht="43" hidden="1" x14ac:dyDescent="0.5">
+    <row r="302" spans="1:5" ht="43" x14ac:dyDescent="0.5">
       <c r="A302" s="1" t="s">
         <v>597</v>
       </c>
@@ -33317,7 +33299,7 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="305" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
+    <row r="305" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A305" s="1" t="s">
         <v>603</v>
       </c>
@@ -33362,7 +33344,7 @@
         <v>2003</v>
       </c>
     </row>
-    <row r="308" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A308" s="1" t="s">
         <v>609</v>
       </c>
@@ -33449,7 +33431,7 @@
         <v>2003</v>
       </c>
     </row>
-    <row r="314" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A314" s="1" t="s">
         <v>621</v>
       </c>
@@ -33718,7 +33700,7 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="333" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
+    <row r="333" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A333" s="1" t="s">
         <v>659</v>
       </c>
@@ -34537,7 +34519,7 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="390" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
+    <row r="390" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A390" s="1" t="s">
         <v>770</v>
       </c>
@@ -35115,7 +35097,7 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="430" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="430" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A430" s="1" t="s">
         <v>850</v>
       </c>
@@ -36410,7 +36392,7 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="521" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
+    <row r="521" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A521" s="1" t="s">
         <v>1031</v>
       </c>
@@ -36727,7 +36709,7 @@
         <v>2012</v>
       </c>
     </row>
-    <row r="543" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="543" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A543" s="1" t="s">
         <v>1071</v>
       </c>
@@ -36744,7 +36726,7 @@
         <v>2015</v>
       </c>
     </row>
-    <row r="544" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="544" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A544" s="1" t="s">
         <v>1071</v>
       </c>
@@ -37123,7 +37105,7 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="570" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="570" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
       <c r="A570" s="1" t="s">
         <v>1124</v>
       </c>
@@ -37659,7 +37641,7 @@
         <v>2012</v>
       </c>
     </row>
-    <row r="607" spans="1:5" ht="43" hidden="1" x14ac:dyDescent="0.5">
+    <row r="607" spans="1:5" ht="43" x14ac:dyDescent="0.5">
       <c r="A607" s="1" t="s">
         <v>1197</v>
       </c>
@@ -38102,7 +38084,7 @@
         <v>2009</v>
       </c>
     </row>
-    <row r="638" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
+    <row r="638" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A638" s="1" t="s">
         <v>1259</v>
       </c>
@@ -38329,7 +38311,7 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="654" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
+    <row r="654" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A654" s="1" t="s">
         <v>1291</v>
       </c>
@@ -38817,7 +38799,7 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="688" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
+    <row r="688" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A688" s="1" t="s">
         <v>1359</v>
       </c>
@@ -38848,7 +38830,7 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="690" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="690" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A690" s="1" t="s">
         <v>1363</v>
       </c>
@@ -38893,7 +38875,7 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="693" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="693" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A693" s="1" t="s">
         <v>1369</v>
       </c>
@@ -39316,7 +39298,7 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="723" spans="1:5" ht="43" hidden="1" x14ac:dyDescent="0.5">
+    <row r="723" spans="1:5" ht="43" x14ac:dyDescent="0.5">
       <c r="A723" s="1" t="s">
         <v>1429</v>
       </c>
@@ -39714,7 +39696,7 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="751" spans="1:5" ht="57.35" hidden="1" x14ac:dyDescent="0.5">
+    <row r="751" spans="1:5" ht="57.35" x14ac:dyDescent="0.5">
       <c r="A751" s="1" t="s">
         <v>1992</v>
       </c>
@@ -40014,7 +39996,7 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="772" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="772" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A772" s="1" t="s">
         <v>1522</v>
       </c>
@@ -40737,7 +40719,7 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="823" spans="1:5" ht="43" hidden="1" x14ac:dyDescent="0.5">
+    <row r="823" spans="1:5" ht="43" x14ac:dyDescent="0.5">
       <c r="A823" s="1" t="s">
         <v>1624</v>
       </c>
@@ -40782,7 +40764,7 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="826" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
+    <row r="826" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A826" s="1" t="s">
         <v>1630</v>
       </c>
@@ -40956,7 +40938,7 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="838" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
+    <row r="838" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A838" s="1" t="s">
         <v>1654</v>
       </c>
@@ -41043,7 +41025,7 @@
         <v>2012</v>
       </c>
     </row>
-    <row r="844" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
+    <row r="844" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A844" s="1" t="s">
         <v>1666</v>
       </c>
@@ -41559,7 +41541,7 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="880" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="880" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A880" s="1" t="s">
         <v>1738</v>
       </c>
@@ -42103,7 +42085,7 @@
         <v>2012</v>
       </c>
     </row>
-    <row r="918" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="918" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
       <c r="A918" s="1" t="s">
         <v>1814</v>
       </c>
@@ -42451,7 +42433,7 @@
         <v>2003</v>
       </c>
     </row>
-    <row r="942" spans="1:5" ht="28.7" hidden="1" x14ac:dyDescent="0.5">
+    <row r="942" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A942" s="1" t="s">
         <v>1862</v>
       </c>
@@ -42510,7 +42492,7 @@
         <v>2003</v>
       </c>
     </row>
-    <row r="946" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="946" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A946" s="1" t="s">
         <v>1870</v>
       </c>
@@ -42653,7 +42635,7 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="956" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="956" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
       <c r="A956" s="1" t="s">
         <v>1890</v>
       </c>
@@ -42967,7 +42949,7 @@
         <v>2012</v>
       </c>
     </row>
-    <row r="978" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="978" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
       <c r="A978" s="1" t="s">
         <v>1934</v>
       </c>
@@ -42998,7 +42980,7 @@
         <v>2010</v>
       </c>
     </row>
-    <row r="980" spans="1:5" hidden="1" x14ac:dyDescent="0.5">
+    <row r="980" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A980" s="1" t="s">
         <v>1938</v>
       </c>
@@ -43808,7 +43790,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E620D641-9DAB-4612-9E35-20F9926442BF}">
-  <dimension ref="A3:B16"/>
+  <dimension ref="A3:B18"/>
   <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="11.29296875" bestFit="1" customWidth="1"/>
@@ -43922,6 +43904,14 @@
     <row r="16" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A16" t="s">
         <v>2024</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A18" t="s">
+        <v>2027</v>
+      </c>
+      <c r="B18">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -43951,7 +43941,7 @@
       <c r="A4" t="s">
         <v>2013</v>
       </c>
-      <c r="B4" s="16">
+      <c r="B4">
         <v>1</v>
       </c>
     </row>
@@ -43959,7 +43949,7 @@
       <c r="A5" t="s">
         <v>2012</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5">
         <v>11</v>
       </c>
     </row>
@@ -43967,7 +43957,7 @@
       <c r="A6" t="s">
         <v>2009</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B6">
         <v>10</v>
       </c>
     </row>
@@ -43975,7 +43965,7 @@
       <c r="A7" t="s">
         <v>2005</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7">
         <v>52</v>
       </c>
     </row>
@@ -43983,7 +43973,7 @@
       <c r="A8" t="s">
         <v>2003</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8">
         <v>10</v>
       </c>
     </row>
@@ -43991,7 +43981,7 @@
       <c r="A9" t="s">
         <v>2004</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9">
         <v>1</v>
       </c>
     </row>
@@ -43999,7 +43989,7 @@
       <c r="A10" t="s">
         <v>2010</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10">
         <v>2</v>
       </c>
     </row>
@@ -44032,1481 +44022,1481 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="143.35" x14ac:dyDescent="0.5">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="14" t="s">
+      <c r="C2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="229.35" x14ac:dyDescent="0.5">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="12" t="s">
+      <c r="C3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="8" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="129" x14ac:dyDescent="0.5">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C4" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="14" t="s">
+      <c r="C4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>2009</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="6" t="s">
         <v>2009</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="157.69999999999999" x14ac:dyDescent="0.5">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="10" t="s">
         <v>1998</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="7" t="s">
         <v>1999</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="12" t="s">
+      <c r="C5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="8" t="s">
         <v>2016</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="186.35" x14ac:dyDescent="0.5">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="C6" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="14" t="s">
+      <c r="C6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="6" t="s">
         <v>2017</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="301" x14ac:dyDescent="0.5">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="C7" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="12" t="s">
+      <c r="C7" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="8" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="57.35" x14ac:dyDescent="0.5">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="C8" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="14" t="s">
+      <c r="C8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="E8" s="6" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="172" x14ac:dyDescent="0.5">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="C9" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="12" t="s">
+      <c r="C9" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>2003</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="8" t="s">
         <v>2003</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="409.6" x14ac:dyDescent="0.5">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="9" t="s">
         <v>2000</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="5" t="s">
         <v>2001</v>
       </c>
-      <c r="C10" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="14" t="s">
+      <c r="C10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>2012</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="E10" s="6" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="186.35" x14ac:dyDescent="0.5">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="10" t="s">
         <v>226</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="C11" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="12" t="s">
+      <c r="C11" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="8" t="s">
         <v>2016</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="243.7" x14ac:dyDescent="0.5">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="C12" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="14" t="s">
+      <c r="C12" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>2012</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="6" t="s">
         <v>2012</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="186.35" x14ac:dyDescent="0.5">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="7" t="s">
         <v>273</v>
       </c>
-      <c r="C13" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="12" t="s">
+      <c r="C13" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="8" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="409.6" x14ac:dyDescent="0.5">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="9" t="s">
         <v>276</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="C14" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="14" t="s">
+      <c r="C14" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="E14" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="215" x14ac:dyDescent="0.5">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="7" t="s">
         <v>293</v>
       </c>
-      <c r="C15" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" s="12" t="s">
+      <c r="C15" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>2012</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="8" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="301" x14ac:dyDescent="0.5">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="9" t="s">
         <v>374</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="5" t="s">
         <v>375</v>
       </c>
-      <c r="C16" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="14" t="s">
+      <c r="C16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>2003</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="E16" s="6" t="s">
         <v>2003</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="143.35" x14ac:dyDescent="0.5">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="10" t="s">
         <v>410</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="7" t="s">
         <v>411</v>
       </c>
-      <c r="C17" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D17" s="12" t="s">
+      <c r="C17" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E17" s="13" t="s">
+      <c r="E17" s="8" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="286.7" x14ac:dyDescent="0.5">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="9" t="s">
         <v>440</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="5" t="s">
         <v>441</v>
       </c>
-      <c r="C18" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D18" s="14" t="s">
+      <c r="C18" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>2003</v>
       </c>
-      <c r="E18" s="15" t="s">
+      <c r="E18" s="6" t="s">
         <v>2003</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="315.35000000000002" x14ac:dyDescent="0.5">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="10" t="s">
         <v>454</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="7" t="s">
         <v>455</v>
       </c>
-      <c r="C19" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D19" s="12" t="s">
+      <c r="C19" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>2003</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="E19" s="8" t="s">
         <v>2003</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="129" x14ac:dyDescent="0.5">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="9" t="s">
         <v>552</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="5" t="s">
         <v>553</v>
       </c>
-      <c r="C20" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D20" s="14" t="s">
+      <c r="C20" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>2009</v>
       </c>
-      <c r="E20" s="15" t="s">
+      <c r="E20" s="6" t="s">
         <v>2009</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="401.35" x14ac:dyDescent="0.5">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="7" t="s">
         <v>598</v>
       </c>
-      <c r="C21" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D21" s="12" t="s">
+      <c r="C21" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="8" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="200.7" x14ac:dyDescent="0.5">
-      <c r="A22" s="17" t="s">
+      <c r="A22" s="9" t="s">
         <v>603</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="5" t="s">
         <v>604</v>
       </c>
-      <c r="C22" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D22" s="14" t="s">
+      <c r="C22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="143.35" x14ac:dyDescent="0.5">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="10" t="s">
         <v>609</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="7" t="s">
         <v>610</v>
       </c>
-      <c r="C23" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D23" s="12" t="s">
+      <c r="C23" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="E23" s="8" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="114.7" x14ac:dyDescent="0.5">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="9" t="s">
         <v>621</v>
       </c>
-      <c r="B24" s="14" t="s">
+      <c r="B24" s="5" t="s">
         <v>622</v>
       </c>
-      <c r="C24" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D24" s="14" t="s">
+      <c r="C24" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E24" s="15" t="s">
+      <c r="E24" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="286.7" x14ac:dyDescent="0.5">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="10" t="s">
         <v>659</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="7" t="s">
         <v>660</v>
       </c>
-      <c r="C25" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D25" s="12" t="s">
+      <c r="C25" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="E25" s="8" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="387" x14ac:dyDescent="0.5">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="9" t="s">
         <v>1983</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="5" t="s">
         <v>1984</v>
       </c>
-      <c r="C26" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D26" s="14" t="s">
+      <c r="C26" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>2009</v>
       </c>
-      <c r="E26" s="15" t="s">
+      <c r="E26" s="6" t="s">
         <v>2009</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="186.35" x14ac:dyDescent="0.5">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="10" t="s">
         <v>663</v>
       </c>
-      <c r="B27" s="12" t="s">
+      <c r="B27" s="7" t="s">
         <v>664</v>
       </c>
-      <c r="C27" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D27" s="12" t="s">
+      <c r="C27" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>2012</v>
       </c>
-      <c r="E27" s="13" t="s">
+      <c r="E27" s="8" t="s">
         <v>2012</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="329.7" x14ac:dyDescent="0.5">
-      <c r="A28" s="17" t="s">
+      <c r="A28" s="9" t="s">
         <v>669</v>
       </c>
-      <c r="B28" s="14" t="s">
+      <c r="B28" s="5" t="s">
         <v>670</v>
       </c>
-      <c r="C28" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D28" s="14" t="s">
+      <c r="C28" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D28" s="5" t="s">
         <v>2012</v>
       </c>
-      <c r="E28" s="15" t="s">
+      <c r="E28" s="6" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="157.69999999999999" x14ac:dyDescent="0.5">
-      <c r="A29" s="18" t="s">
+      <c r="A29" s="10" t="s">
         <v>685</v>
       </c>
-      <c r="B29" s="12" t="s">
+      <c r="B29" s="7" t="s">
         <v>686</v>
       </c>
-      <c r="C29" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D29" s="12" t="s">
+      <c r="C29" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" s="7" t="s">
         <v>2003</v>
       </c>
-      <c r="E29" s="13" t="s">
+      <c r="E29" s="8" t="s">
         <v>2003</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="409.6" x14ac:dyDescent="0.5">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="9" t="s">
         <v>1985</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="B30" s="5" t="s">
         <v>705</v>
       </c>
-      <c r="C30" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D30" s="14" t="s">
+      <c r="C30" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>2010</v>
       </c>
-      <c r="E30" s="15" t="s">
+      <c r="E30" s="6" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="229.35" x14ac:dyDescent="0.5">
-      <c r="A31" s="18" t="s">
+      <c r="A31" s="10" t="s">
         <v>712</v>
       </c>
-      <c r="B31" s="12" t="s">
+      <c r="B31" s="7" t="s">
         <v>713</v>
       </c>
-      <c r="C31" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D31" s="12" t="s">
+      <c r="C31" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D31" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="E31" s="8" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="344" x14ac:dyDescent="0.5">
-      <c r="A32" s="17" t="s">
+      <c r="A32" s="9" t="s">
         <v>770</v>
       </c>
-      <c r="B32" s="14" t="s">
+      <c r="B32" s="5" t="s">
         <v>771</v>
       </c>
-      <c r="C32" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D32" s="14" t="s">
+      <c r="C32" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D32" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E32" s="15" t="s">
+      <c r="E32" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="358.35" x14ac:dyDescent="0.5">
-      <c r="A33" s="18" t="s">
+      <c r="A33" s="10" t="s">
         <v>778</v>
       </c>
-      <c r="B33" s="12" t="s">
+      <c r="B33" s="7" t="s">
         <v>779</v>
       </c>
-      <c r="C33" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D33" s="12" t="s">
+      <c r="C33" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D33" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E33" s="13" t="s">
+      <c r="E33" s="8" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="409.6" x14ac:dyDescent="0.5">
-      <c r="A34" s="17" t="s">
+      <c r="A34" s="9" t="s">
         <v>808</v>
       </c>
-      <c r="B34" s="14" t="s">
+      <c r="B34" s="5" t="s">
         <v>809</v>
       </c>
-      <c r="C34" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D34" s="14" t="s">
+      <c r="C34" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>2012</v>
       </c>
-      <c r="E34" s="15" t="s">
+      <c r="E34" s="6" t="s">
         <v>2012</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="200.7" x14ac:dyDescent="0.5">
-      <c r="A35" s="18" t="s">
+      <c r="A35" s="10" t="s">
         <v>816</v>
       </c>
-      <c r="B35" s="12" t="s">
+      <c r="B35" s="7" t="s">
         <v>817</v>
       </c>
-      <c r="C35" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D35" s="12" t="s">
+      <c r="C35" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E35" s="13" t="s">
+      <c r="E35" s="8" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="200.7" x14ac:dyDescent="0.5">
-      <c r="A36" s="17" t="s">
+      <c r="A36" s="9" t="s">
         <v>826</v>
       </c>
-      <c r="B36" s="14" t="s">
+      <c r="B36" s="5" t="s">
         <v>827</v>
       </c>
-      <c r="C36" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D36" s="14" t="s">
+      <c r="C36" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E36" s="15" t="s">
+      <c r="E36" s="6" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="129" x14ac:dyDescent="0.5">
-      <c r="A37" s="18" t="s">
+      <c r="A37" s="10" t="s">
         <v>830</v>
       </c>
-      <c r="B37" s="12" t="s">
+      <c r="B37" s="7" t="s">
         <v>831</v>
       </c>
-      <c r="C37" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D37" s="12" t="s">
+      <c r="C37" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" s="7" t="s">
         <v>2009</v>
       </c>
-      <c r="E37" s="13" t="s">
+      <c r="E37" s="8" t="s">
         <v>2009</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="114.7" x14ac:dyDescent="0.5">
-      <c r="A38" s="17" t="s">
+      <c r="A38" s="9" t="s">
         <v>850</v>
       </c>
-      <c r="B38" s="14" t="s">
+      <c r="B38" s="5" t="s">
         <v>851</v>
       </c>
-      <c r="C38" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D38" s="14" t="s">
+      <c r="C38" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" s="5" t="s">
         <v>2012</v>
       </c>
-      <c r="E38" s="15" t="s">
+      <c r="E38" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="344" x14ac:dyDescent="0.5">
-      <c r="A39" s="18" t="s">
+      <c r="A39" s="10" t="s">
         <v>938</v>
       </c>
-      <c r="B39" s="12" t="s">
+      <c r="B39" s="7" t="s">
         <v>939</v>
       </c>
-      <c r="C39" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D39" s="12" t="s">
+      <c r="C39" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" s="7" t="s">
         <v>2009</v>
       </c>
-      <c r="E39" s="13" t="s">
+      <c r="E39" s="8" t="s">
         <v>2009</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="129" x14ac:dyDescent="0.5">
-      <c r="A40" s="17" t="s">
+      <c r="A40" s="9" t="s">
         <v>948</v>
       </c>
-      <c r="B40" s="14" t="s">
+      <c r="B40" s="5" t="s">
         <v>949</v>
       </c>
-      <c r="C40" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D40" s="14" t="s">
+      <c r="C40" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D40" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E40" s="15" t="s">
+      <c r="E40" s="6" t="s">
         <v>2017</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="301" x14ac:dyDescent="0.5">
-      <c r="A41" s="18" t="s">
+      <c r="A41" s="10" t="s">
         <v>952</v>
       </c>
-      <c r="B41" s="12" t="s">
+      <c r="B41" s="7" t="s">
         <v>953</v>
       </c>
-      <c r="C41" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D41" s="12" t="s">
+      <c r="C41" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D41" s="7" t="s">
         <v>2012</v>
       </c>
-      <c r="E41" s="13" t="s">
+      <c r="E41" s="8" t="s">
         <v>2012</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="229.35" x14ac:dyDescent="0.5">
-      <c r="A42" s="17" t="s">
+      <c r="A42" s="9" t="s">
         <v>970</v>
       </c>
-      <c r="B42" s="14" t="s">
+      <c r="B42" s="5" t="s">
         <v>971</v>
       </c>
-      <c r="C42" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D42" s="14" t="s">
+      <c r="C42" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D42" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E42" s="15" t="s">
+      <c r="E42" s="6" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="409.6" x14ac:dyDescent="0.5">
-      <c r="A43" s="18" t="s">
+      <c r="A43" s="10" t="s">
         <v>982</v>
       </c>
-      <c r="B43" s="12" t="s">
+      <c r="B43" s="7" t="s">
         <v>983</v>
       </c>
-      <c r="C43" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D43" s="12" t="s">
+      <c r="C43" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D43" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E43" s="13" t="s">
+      <c r="E43" s="8" t="s">
         <v>2009</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="315.35000000000002" x14ac:dyDescent="0.5">
-      <c r="A44" s="17" t="s">
+      <c r="A44" s="9" t="s">
         <v>1031</v>
       </c>
-      <c r="B44" s="14" t="s">
+      <c r="B44" s="5" t="s">
         <v>1032</v>
       </c>
-      <c r="C44" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D44" s="14" t="s">
+      <c r="C44" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D44" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E44" s="15" t="s">
+      <c r="E44" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="286.7" x14ac:dyDescent="0.5">
-      <c r="A45" s="18" t="s">
+      <c r="A45" s="10" t="s">
         <v>1045</v>
       </c>
-      <c r="B45" s="12" t="s">
+      <c r="B45" s="7" t="s">
         <v>1046</v>
       </c>
-      <c r="C45" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D45" s="12" t="s">
+      <c r="C45" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D45" s="7" t="s">
         <v>2003</v>
       </c>
-      <c r="E45" s="13" t="s">
+      <c r="E45" s="8" t="s">
         <v>2003</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="129" x14ac:dyDescent="0.5">
-      <c r="A46" s="17" t="s">
+      <c r="A46" s="9" t="s">
         <v>1071</v>
       </c>
-      <c r="B46" s="14" t="s">
+      <c r="B46" s="5" t="s">
         <v>1072</v>
       </c>
-      <c r="C46" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D46" s="14" t="s">
+      <c r="C46" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D46" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E46" s="15" t="s">
+      <c r="E46" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="129" x14ac:dyDescent="0.5">
-      <c r="A47" s="18" t="s">
+      <c r="A47" s="10" t="s">
         <v>1071</v>
       </c>
-      <c r="B47" s="12" t="s">
+      <c r="B47" s="7" t="s">
         <v>1073</v>
       </c>
-      <c r="C47" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D47" s="12" t="s">
+      <c r="C47" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D47" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E47" s="13" t="s">
+      <c r="E47" s="8" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="258" x14ac:dyDescent="0.5">
-      <c r="A48" s="17" t="s">
+      <c r="A48" s="9" t="s">
         <v>1084</v>
       </c>
-      <c r="B48" s="14" t="s">
+      <c r="B48" s="5" t="s">
         <v>1085</v>
       </c>
-      <c r="C48" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D48" s="14" t="s">
+      <c r="C48" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D48" s="5" t="s">
         <v>2012</v>
       </c>
-      <c r="E48" s="15" t="s">
+      <c r="E48" s="6" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="172" x14ac:dyDescent="0.5">
-      <c r="A49" s="18" t="s">
+      <c r="A49" s="10" t="s">
         <v>1086</v>
       </c>
-      <c r="B49" s="12" t="s">
+      <c r="B49" s="7" t="s">
         <v>1087</v>
       </c>
-      <c r="C49" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D49" s="12" t="s">
+      <c r="C49" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D49" s="7" t="s">
         <v>2013</v>
       </c>
-      <c r="E49" s="13" t="s">
+      <c r="E49" s="8" t="s">
         <v>2012</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="286.7" x14ac:dyDescent="0.5">
-      <c r="A50" s="17" t="s">
+      <c r="A50" s="9" t="s">
         <v>1108</v>
       </c>
-      <c r="B50" s="14" t="s">
+      <c r="B50" s="5" t="s">
         <v>1109</v>
       </c>
-      <c r="C50" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D50" s="14" t="s">
+      <c r="C50" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D50" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E50" s="15" t="s">
+      <c r="E50" s="6" t="s">
         <v>2012</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="243.7" x14ac:dyDescent="0.5">
-      <c r="A51" s="18" t="s">
+      <c r="A51" s="10" t="s">
         <v>1116</v>
       </c>
-      <c r="B51" s="12" t="s">
+      <c r="B51" s="7" t="s">
         <v>1117</v>
       </c>
-      <c r="C51" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D51" s="12" t="s">
+      <c r="C51" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51" s="7" t="s">
         <v>2009</v>
       </c>
-      <c r="E51" s="13" t="s">
+      <c r="E51" s="8" t="s">
         <v>2009</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="100.35" x14ac:dyDescent="0.5">
-      <c r="A52" s="17" t="s">
+      <c r="A52" s="9" t="s">
         <v>1142</v>
       </c>
-      <c r="B52" s="14" t="s">
+      <c r="B52" s="5" t="s">
         <v>1143</v>
       </c>
-      <c r="C52" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D52" s="14" t="s">
+      <c r="C52" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D52" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E52" s="15" t="s">
+      <c r="E52" s="6" t="s">
         <v>2010</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="409.6" x14ac:dyDescent="0.5">
-      <c r="A53" s="18" t="s">
+      <c r="A53" s="10" t="s">
         <v>1144</v>
       </c>
-      <c r="B53" s="12" t="s">
+      <c r="B53" s="7" t="s">
         <v>1145</v>
       </c>
-      <c r="C53" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D53" s="12" t="s">
+      <c r="C53" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D53" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E53" s="13" t="s">
+      <c r="E53" s="8" t="s">
         <v>2017</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="200.7" x14ac:dyDescent="0.5">
-      <c r="A54" s="17" t="s">
+      <c r="A54" s="9" t="s">
         <v>1180</v>
       </c>
-      <c r="B54" s="14" t="s">
+      <c r="B54" s="5" t="s">
         <v>1181</v>
       </c>
-      <c r="C54" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D54" s="14" t="s">
+      <c r="C54" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D54" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E54" s="15" t="s">
+      <c r="E54" s="6" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="114.7" x14ac:dyDescent="0.5">
-      <c r="A55" s="18" t="s">
+      <c r="A55" s="10" t="s">
         <v>1182</v>
       </c>
-      <c r="B55" s="12" t="s">
+      <c r="B55" s="7" t="s">
         <v>1183</v>
       </c>
-      <c r="C55" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D55" s="12" t="s">
+      <c r="C55" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D55" s="7" t="s">
         <v>2009</v>
       </c>
-      <c r="E55" s="13" t="s">
+      <c r="E55" s="8" t="s">
         <v>2009</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="100.35" x14ac:dyDescent="0.5">
-      <c r="A56" s="17" t="s">
+      <c r="A56" s="9" t="s">
         <v>1184</v>
       </c>
-      <c r="B56" s="14" t="s">
+      <c r="B56" s="5" t="s">
         <v>1185</v>
       </c>
-      <c r="C56" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D56" s="14" t="s">
+      <c r="C56" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D56" s="5" t="s">
         <v>2012</v>
       </c>
-      <c r="E56" s="15" t="s">
+      <c r="E56" s="6" t="s">
         <v>2012</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="86" x14ac:dyDescent="0.5">
-      <c r="A57" s="18" t="s">
+      <c r="A57" s="10" t="s">
         <v>1245</v>
       </c>
-      <c r="B57" s="12" t="s">
+      <c r="B57" s="7" t="s">
         <v>1246</v>
       </c>
-      <c r="C57" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D57" s="12" t="s">
+      <c r="C57" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D57" s="7" t="s">
         <v>2009</v>
       </c>
-      <c r="E57" s="13" t="s">
+      <c r="E57" s="8" t="s">
         <v>2009</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="157.69999999999999" x14ac:dyDescent="0.5">
-      <c r="A58" s="17" t="s">
+      <c r="A58" s="9" t="s">
         <v>1253</v>
       </c>
-      <c r="B58" s="14" t="s">
+      <c r="B58" s="5" t="s">
         <v>1254</v>
       </c>
-      <c r="C58" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D58" s="14" t="s">
+      <c r="C58" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D58" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E58" s="15" t="s">
+      <c r="E58" s="6" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="258" x14ac:dyDescent="0.5">
-      <c r="A59" s="18" t="s">
+      <c r="A59" s="10" t="s">
         <v>1259</v>
       </c>
-      <c r="B59" s="12" t="s">
+      <c r="B59" s="7" t="s">
         <v>1260</v>
       </c>
-      <c r="C59" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D59" s="12" t="s">
+      <c r="C59" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D59" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E59" s="13" t="s">
+      <c r="E59" s="8" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="243.7" x14ac:dyDescent="0.5">
-      <c r="A60" s="17" t="s">
+      <c r="A60" s="9" t="s">
         <v>1291</v>
       </c>
-      <c r="B60" s="14" t="s">
+      <c r="B60" s="5" t="s">
         <v>1292</v>
       </c>
-      <c r="C60" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D60" s="14" t="s">
+      <c r="C60" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D60" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E60" s="15" t="s">
+      <c r="E60" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="301" x14ac:dyDescent="0.5">
-      <c r="A61" s="18" t="s">
+      <c r="A61" s="10" t="s">
         <v>1335</v>
       </c>
-      <c r="B61" s="12" t="s">
+      <c r="B61" s="7" t="s">
         <v>1336</v>
       </c>
-      <c r="C61" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D61" s="12" t="s">
+      <c r="C61" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D61" s="7" t="s">
         <v>2009</v>
       </c>
-      <c r="E61" s="13" t="s">
+      <c r="E61" s="8" t="s">
         <v>2009</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="129" x14ac:dyDescent="0.5">
-      <c r="A62" s="17" t="s">
+      <c r="A62" s="9" t="s">
         <v>1341</v>
       </c>
-      <c r="B62" s="14" t="s">
+      <c r="B62" s="5" t="s">
         <v>1342</v>
       </c>
-      <c r="C62" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D62" s="14" t="s">
+      <c r="C62" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D62" s="5" t="s">
         <v>2003</v>
       </c>
-      <c r="E62" s="15" t="s">
+      <c r="E62" s="6" t="s">
         <v>2003</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="301" x14ac:dyDescent="0.5">
-      <c r="A63" s="18" t="s">
+      <c r="A63" s="10" t="s">
         <v>1359</v>
       </c>
-      <c r="B63" s="12" t="s">
+      <c r="B63" s="7" t="s">
         <v>1360</v>
       </c>
-      <c r="C63" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D63" s="12" t="s">
+      <c r="C63" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D63" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E63" s="13" t="s">
+      <c r="E63" s="8" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="100.35" x14ac:dyDescent="0.5">
-      <c r="A64" s="17" t="s">
+      <c r="A64" s="9" t="s">
         <v>1363</v>
       </c>
-      <c r="B64" s="14" t="s">
+      <c r="B64" s="5" t="s">
         <v>1364</v>
       </c>
-      <c r="C64" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D64" s="14" t="s">
+      <c r="C64" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E64" s="15" t="s">
+      <c r="E64" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="100.35" x14ac:dyDescent="0.5">
-      <c r="A65" s="18" t="s">
+      <c r="A65" s="10" t="s">
         <v>1369</v>
       </c>
-      <c r="B65" s="12" t="s">
+      <c r="B65" s="7" t="s">
         <v>1370</v>
       </c>
-      <c r="C65" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D65" s="12" t="s">
+      <c r="C65" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E65" s="13" t="s">
+      <c r="E65" s="8" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="401.35" x14ac:dyDescent="0.5">
-      <c r="A66" s="17" t="s">
+      <c r="A66" s="9" t="s">
         <v>1429</v>
       </c>
-      <c r="B66" s="14" t="s">
+      <c r="B66" s="5" t="s">
         <v>1430</v>
       </c>
-      <c r="C66" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D66" s="14" t="s">
+      <c r="C66" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D66" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E66" s="15" t="s">
+      <c r="E66" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="215" x14ac:dyDescent="0.5">
-      <c r="A67" s="18" t="s">
+      <c r="A67" s="10" t="s">
         <v>1453</v>
       </c>
-      <c r="B67" s="12" t="s">
+      <c r="B67" s="7" t="s">
         <v>1454</v>
       </c>
-      <c r="C67" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D67" s="12" t="s">
+      <c r="C67" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D67" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E67" s="13" t="s">
+      <c r="E67" s="8" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="409.6" x14ac:dyDescent="0.5">
-      <c r="A68" s="17" t="s">
+      <c r="A68" s="9" t="s">
         <v>1992</v>
       </c>
-      <c r="B68" s="14" t="s">
+      <c r="B68" s="5" t="s">
         <v>1993</v>
       </c>
-      <c r="C68" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D68" s="14" t="s">
+      <c r="C68" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D68" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E68" s="15" t="s">
+      <c r="E68" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="315.35000000000002" x14ac:dyDescent="0.5">
-      <c r="A69" s="18" t="s">
+      <c r="A69" s="10" t="s">
         <v>1500</v>
       </c>
-      <c r="B69" s="12" t="s">
+      <c r="B69" s="7" t="s">
         <v>1501</v>
       </c>
-      <c r="C69" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D69" s="12" t="s">
+      <c r="C69" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D69" s="7" t="s">
         <v>2009</v>
       </c>
-      <c r="E69" s="13" t="s">
+      <c r="E69" s="8" t="s">
         <v>2009</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="71.7" x14ac:dyDescent="0.5">
-      <c r="A70" s="17" t="s">
+      <c r="A70" s="9" t="s">
         <v>1522</v>
       </c>
-      <c r="B70" s="14" t="s">
+      <c r="B70" s="5" t="s">
         <v>1523</v>
       </c>
-      <c r="C70" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D70" s="14" t="s">
+      <c r="C70" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D70" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E70" s="15" t="s">
+      <c r="E70" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="229.35" x14ac:dyDescent="0.5">
-      <c r="A71" s="18" t="s">
+      <c r="A71" s="10" t="s">
         <v>1560</v>
       </c>
-      <c r="B71" s="12" t="s">
+      <c r="B71" s="7" t="s">
         <v>1561</v>
       </c>
-      <c r="C71" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D71" s="12" t="s">
+      <c r="C71" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D71" s="7" t="s">
         <v>2010</v>
       </c>
-      <c r="E71" s="13" t="s">
+      <c r="E71" s="8" t="s">
         <v>2010</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="129" x14ac:dyDescent="0.5">
-      <c r="A72" s="17" t="s">
+      <c r="A72" s="9" t="s">
         <v>1604</v>
       </c>
-      <c r="B72" s="14" t="s">
+      <c r="B72" s="5" t="s">
         <v>1605</v>
       </c>
-      <c r="C72" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D72" s="14" t="s">
+      <c r="C72" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D72" s="5" t="s">
         <v>2003</v>
       </c>
-      <c r="E72" s="15" t="s">
+      <c r="E72" s="6" t="s">
         <v>2003</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="315.35000000000002" x14ac:dyDescent="0.5">
-      <c r="A73" s="18" t="s">
+      <c r="A73" s="10" t="s">
         <v>1624</v>
       </c>
-      <c r="B73" s="12" t="s">
+      <c r="B73" s="7" t="s">
         <v>1625</v>
       </c>
-      <c r="C73" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D73" s="12" t="s">
+      <c r="C73" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D73" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E73" s="13" t="s">
+      <c r="E73" s="8" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="200.7" x14ac:dyDescent="0.5">
-      <c r="A74" s="17" t="s">
+      <c r="A74" s="9" t="s">
         <v>1630</v>
       </c>
-      <c r="B74" s="14" t="s">
+      <c r="B74" s="5" t="s">
         <v>1631</v>
       </c>
-      <c r="C74" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D74" s="14" t="s">
+      <c r="C74" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D74" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E74" s="15" t="s">
+      <c r="E74" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="200.7" x14ac:dyDescent="0.5">
-      <c r="A75" s="18" t="s">
+      <c r="A75" s="10" t="s">
         <v>1654</v>
       </c>
-      <c r="B75" s="12" t="s">
+      <c r="B75" s="7" t="s">
         <v>1655</v>
       </c>
-      <c r="C75" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D75" s="12" t="s">
+      <c r="C75" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D75" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E75" s="13" t="s">
+      <c r="E75" s="8" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="200.7" x14ac:dyDescent="0.5">
-      <c r="A76" s="17" t="s">
+      <c r="A76" s="9" t="s">
         <v>1666</v>
       </c>
-      <c r="B76" s="14" t="s">
+      <c r="B76" s="5" t="s">
         <v>1667</v>
       </c>
-      <c r="C76" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D76" s="14" t="s">
+      <c r="C76" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D76" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E76" s="15" t="s">
+      <c r="E76" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="114.7" x14ac:dyDescent="0.5">
-      <c r="A77" s="18" t="s">
+      <c r="A77" s="10" t="s">
         <v>1680</v>
       </c>
-      <c r="B77" s="12" t="s">
+      <c r="B77" s="7" t="s">
         <v>1681</v>
       </c>
-      <c r="C77" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D77" s="12" t="s">
+      <c r="C77" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D77" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E77" s="13" t="s">
+      <c r="E77" s="8" t="s">
         <v>2017</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="172" x14ac:dyDescent="0.5">
-      <c r="A78" s="17" t="s">
+      <c r="A78" s="9" t="s">
         <v>1684</v>
       </c>
-      <c r="B78" s="14" t="s">
+      <c r="B78" s="5" t="s">
         <v>1685</v>
       </c>
-      <c r="C78" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D78" s="14" t="s">
+      <c r="C78" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D78" s="5" t="s">
         <v>2003</v>
       </c>
-      <c r="E78" s="15" t="s">
+      <c r="E78" s="6" t="s">
         <v>2003</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="157.69999999999999" x14ac:dyDescent="0.5">
-      <c r="A79" s="18" t="s">
+      <c r="A79" s="10" t="s">
         <v>1738</v>
       </c>
-      <c r="B79" s="12" t="s">
+      <c r="B79" s="7" t="s">
         <v>1739</v>
       </c>
-      <c r="C79" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D79" s="12" t="s">
+      <c r="C79" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D79" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E79" s="13" t="s">
+      <c r="E79" s="8" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="114.7" x14ac:dyDescent="0.5">
-      <c r="A80" s="17" t="s">
+      <c r="A80" s="9" t="s">
         <v>1754</v>
       </c>
-      <c r="B80" s="14" t="s">
+      <c r="B80" s="5" t="s">
         <v>1755</v>
       </c>
-      <c r="C80" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D80" s="14" t="s">
+      <c r="C80" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D80" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E80" s="15" t="s">
+      <c r="E80" s="6" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="81" spans="1:5" ht="200.7" x14ac:dyDescent="0.5">
-      <c r="A81" s="18" t="s">
+      <c r="A81" s="10" t="s">
         <v>1758</v>
       </c>
-      <c r="B81" s="12" t="s">
+      <c r="B81" s="7" t="s">
         <v>1759</v>
       </c>
-      <c r="C81" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D81" s="12" t="s">
+      <c r="C81" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D81" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E81" s="13" t="s">
+      <c r="E81" s="8" t="s">
         <v>2017</v>
       </c>
     </row>
     <row r="82" spans="1:5" ht="215" x14ac:dyDescent="0.5">
-      <c r="A82" s="17" t="s">
+      <c r="A82" s="9" t="s">
         <v>1820</v>
       </c>
-      <c r="B82" s="14" t="s">
+      <c r="B82" s="5" t="s">
         <v>1821</v>
       </c>
-      <c r="C82" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D82" s="14" t="s">
+      <c r="C82" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D82" s="5" t="s">
         <v>2012</v>
       </c>
-      <c r="E82" s="15" t="s">
+      <c r="E82" s="6" t="s">
         <v>2012</v>
       </c>
     </row>
     <row r="83" spans="1:5" ht="57.35" x14ac:dyDescent="0.5">
-      <c r="A83" s="18" t="s">
+      <c r="A83" s="10" t="s">
         <v>1828</v>
       </c>
-      <c r="B83" s="12" t="s">
+      <c r="B83" s="7" t="s">
         <v>1829</v>
       </c>
-      <c r="C83" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D83" s="12" t="s">
+      <c r="C83" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83" s="7" t="s">
         <v>2003</v>
       </c>
-      <c r="E83" s="13" t="s">
+      <c r="E83" s="8" t="s">
         <v>2003</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="143.35" x14ac:dyDescent="0.5">
-      <c r="A84" s="17" t="s">
+      <c r="A84" s="9" t="s">
         <v>1852</v>
       </c>
-      <c r="B84" s="14" t="s">
+      <c r="B84" s="5" t="s">
         <v>1853</v>
       </c>
-      <c r="C84" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D84" s="14" t="s">
+      <c r="C84" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D84" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E84" s="15" t="s">
+      <c r="E84" s="6" t="s">
         <v>2018</v>
       </c>
     </row>
     <row r="85" spans="1:5" ht="186.35" x14ac:dyDescent="0.5">
-      <c r="A85" s="18" t="s">
+      <c r="A85" s="10" t="s">
         <v>1900</v>
       </c>
-      <c r="B85" s="12" t="s">
+      <c r="B85" s="7" t="s">
         <v>1901</v>
       </c>
-      <c r="C85" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D85" s="12" t="s">
+      <c r="C85" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D85" s="7" t="s">
         <v>2004</v>
       </c>
-      <c r="E85" s="13" t="s">
+      <c r="E85" s="8" t="s">
         <v>2012</v>
       </c>
     </row>
     <row r="86" spans="1:5" ht="28.7" x14ac:dyDescent="0.5">
-      <c r="A86" s="17" t="s">
+      <c r="A86" s="9" t="s">
         <v>1938</v>
       </c>
-      <c r="B86" s="14" t="s">
+      <c r="B86" s="5" t="s">
         <v>1939</v>
       </c>
-      <c r="C86" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D86" s="14" t="s">
+      <c r="C86" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D86" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E86" s="15" t="s">
+      <c r="E86" s="6" t="s">
         <v>2015</v>
       </c>
     </row>
     <row r="87" spans="1:5" ht="43" x14ac:dyDescent="0.5">
-      <c r="A87" s="18" t="s">
+      <c r="A87" s="10" t="s">
         <v>1944</v>
       </c>
-      <c r="B87" s="12" t="s">
+      <c r="B87" s="7" t="s">
         <v>1945</v>
       </c>
-      <c r="C87" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D87" s="12" t="s">
+      <c r="C87" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D87" s="7" t="s">
         <v>2005</v>
       </c>
-      <c r="E87" s="13" t="s">
+      <c r="E87" s="8" t="s">
         <v>2012</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="43" x14ac:dyDescent="0.5">
-      <c r="A88" s="17" t="s">
+      <c r="A88" s="9" t="s">
         <v>1980</v>
       </c>
-      <c r="B88" s="14" t="s">
+      <c r="B88" s="5" t="s">
         <v>1981</v>
       </c>
-      <c r="C88" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D88" s="14" t="s">
+      <c r="C88" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D88" s="5" t="s">
         <v>2005</v>
       </c>
-      <c r="E88" s="15" t="s">
+      <c r="E88" s="6" t="s">
         <v>2012</v>
       </c>
     </row>

</xml_diff>